<commit_message>
feat(phase1): enforce seed URL compliance
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/strategy/Pro-Exteriors_GBP-Curation_April-2026.xlsx
+++ b/strategy/Pro-Exteriors_GBP-Curation_April-2026.xlsx
@@ -5581,7 +5581,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -5701,17 +5701,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>/residential/</t>
+          <t>/residential-roofing/</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -5776,7 +5776,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -6101,7 +6101,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -6221,12 +6221,17 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>/locations/denver/</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -6281,12 +6286,17 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>/locations/wichita/</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -6341,12 +6351,17 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>/locations/kansas-city/</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -6401,12 +6416,17 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>/locations/atlanta/</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -6461,17 +6481,17 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>/commercial-roofing/tpo-roofing-systems/</t>
+          <t>/commercial-roofing/tpo/</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -6536,7 +6556,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -6601,7 +6621,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -6666,7 +6686,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -6731,7 +6751,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -6796,7 +6816,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -6851,17 +6871,17 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>/residential/asphalt-shingles/</t>
+          <t>/residential-roofing/asphalt-shingles/</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -6916,17 +6936,17 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>/residential/roof-replacement/</t>
+          <t>/residential-roofing/replacement/</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -6981,12 +7001,17 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>/residential-roofing/inspection/</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -7041,12 +7066,17 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>/residential-roofing/emergency/</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -7101,17 +7131,17 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>/residential/metal-roofing/</t>
+          <t>/residential-roofing/metal/</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -7166,17 +7196,17 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>/residential/storm-damage-repair/</t>
+          <t>/residential-roofing/storm-damage/</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -7231,12 +7261,17 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>/commercial-roofing/dallas/</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -7291,12 +7326,17 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>/commercial-roofing/fort-worth/</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -7351,12 +7391,17 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>/commercial-roofing/plano/</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -7411,12 +7456,17 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>/commercial-roofing/frisco/</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -7471,12 +7521,17 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>/residential-roofing/dallas/</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -7531,12 +7586,17 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>/residential-roofing/fort-worth/</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -7591,12 +7651,17 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>/residential-roofing/highland-park/</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -7651,12 +7716,17 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>/residential-roofing/southlake/</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -7711,12 +7781,17 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>/contact/commercial/</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -7771,12 +7846,17 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>/contact/residential/inspection/</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -7831,12 +7911,17 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>/contact/emergency/</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -7891,17 +7976,17 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>/thank-you/</t>
+          <t>/thank-you/commercial/</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -7956,17 +8041,17 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>/thank-you/</t>
+          <t>/thank-you/residential/</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -8031,7 +8116,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -8096,7 +8181,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -8151,12 +8236,17 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>/about/certifications/</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -8221,7 +8311,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -8286,7 +8376,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -8351,7 +8441,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -8416,7 +8506,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -8481,7 +8571,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -8546,7 +8636,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -8611,7 +8701,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -8666,17 +8756,17 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>/privacy-policy/</t>
+          <t>/privacy/</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -8741,7 +8831,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -8806,7 +8896,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -8871,7 +8961,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -8926,17 +9016,17 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>/sitemap-index.xml</t>
+          <t>/sitemap.xml</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -8991,12 +9081,17 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>/robots.txt</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -9051,17 +9146,17 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Published noncanonical alternate</t>
+          <t>Published exact</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>/404.html</t>
+          <t>/404/</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Build emits a different URL than the Phase 1/GBP plan. Align route or update plan intentionally.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -9126,7 +9221,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -9191,7 +9286,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -9256,7 +9351,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -9321,7 +9416,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -9386,7 +9481,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -9451,7 +9546,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -9516,7 +9611,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -9581,7 +9676,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -9646,7 +9741,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Current Astro build emits this URL.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -9701,12 +9796,17 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Missing from current build</t>
+          <t>Published exact</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>/residential-roofing/twin-creeks-allen/</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Phase 0 URL is planned in workbook but no matching route exists in verified dist output.</t>
+          <t>Current Astro build emits this Phase 0 URL and audit:gbp-plan verifies it.</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -23598,7 +23698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="43" min="1" max="1"/>
@@ -23656,7 +23756,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="64" t="inlineStr">
         <is>
@@ -23739,7 +23838,6 @@
         <v>102</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="65" t="inlineStr">
         <is>
@@ -27000,7 +27098,6 @@
         </is>
       </c>
     </row>
-    <row r="83"/>
     <row r="84">
       <c r="A84" s="65" t="inlineStr">
         <is>
@@ -27385,7 +27482,6 @@
         </is>
       </c>
     </row>
-    <row r="115"/>
     <row r="116">
       <c r="A116" s="65" t="inlineStr">
         <is>
@@ -27456,7 +27552,6 @@
         </is>
       </c>
     </row>
-    <row r="120"/>
     <row r="121">
       <c r="A121" s="65" t="inlineStr">
         <is>
@@ -27487,6 +27582,28 @@
         </is>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Phase 1 Seed closeout</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>npm run build; npm run audit:gbp-plan</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>66 Phase 0 URLs published exact; build chain includes audit:gbp-plan.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>